<commit_message>
Replace Maps URL column with Address, seed Dad's Barbershop as row 3
Swap the Maps URL column for an Address column (more useful at a glance
than a link) and pre-fill row 3 with everything we know about Dad's
Barbershop: contact Austin, phone, email, address, Facebook + Fresha
presence, status = Won — In Progress. Refreshed the Reference sheet
instructions accordingly.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012PjrxYX9YbzcxAV8ycTXXJ
</commit_message>
<xml_diff>
--- a/tools/website-pipeline.xlsx
+++ b/tools/website-pipeline.xlsx
@@ -311,22 +311,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>template</author>
-  </authors>
-  <commentList>
-    <comment ref="A3" authorId="0" shapeId="0">
-      <text>
-        <t>This is a sample row showing the expected format.
-Delete this row before you start entering real leads.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -625,7 +609,7 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -709,7 +693,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Maps URL</t>
+          <t>Address</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
@@ -821,117 +805,77 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>EXAMPLE — Corner Cafe</t>
+          <t>Dad's Barbershop</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Sam Reid</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>(306) 555-0142</t>
+          <t>(306) 229-0597</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>sam@cornercafe.example</t>
+          <t>dadsbarbershop306@gmail.com</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Cafe</t>
+          <t>Barbershop</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Warman, SK</t>
+          <t>Martensville, SK</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>https://maps.google.com/?cid=EXAMPLE</t>
+          <t>402 1 Avenue South, Martensville, SK</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Facebook only</t>
+          <t>Facebook + Fresha booking</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>Maps scan</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="n">
-        <v>46220</v>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>46221</v>
-      </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>46224</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>46229</v>
-      </c>
+          <t>Own client</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="n"/>
+      <c r="K3" s="8" t="n"/>
+      <c r="L3" s="7" t="n"/>
+      <c r="M3" s="8" t="n"/>
+      <c r="N3" s="8" t="n"/>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>Interested</t>
-        </is>
-      </c>
-      <c r="P3" s="7" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="Q3" s="9" t="n">
-        <v>650</v>
-      </c>
-      <c r="R3" s="9" t="n">
-        <v>200</v>
-      </c>
+          <t>Won — In Progress</t>
+        </is>
+      </c>
+      <c r="P3" s="7" t="n"/>
+      <c r="Q3" s="9" t="n"/>
+      <c r="R3" s="9" t="n"/>
       <c r="S3" s="9">
         <f>IF(Q3="","",Q3-IF(R3="",0,R3))</f>
         <v/>
       </c>
-      <c r="T3" s="8" t="n">
-        <v>46230</v>
-      </c>
-      <c r="U3" s="8" t="n">
-        <v>46240</v>
-      </c>
+      <c r="T3" s="8" t="n"/>
+      <c r="U3" s="8" t="n"/>
       <c r="V3" s="8" t="n"/>
-      <c r="W3" s="7" t="inlineStr"/>
-      <c r="X3" s="10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="Y3" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Z3" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="AA3" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="W3" s="7" t="n"/>
+      <c r="X3" s="10" t="n"/>
+      <c r="Y3" s="10" t="n"/>
+      <c r="Z3" s="10" t="n"/>
+      <c r="AA3" s="10" t="n"/>
       <c r="AB3" s="7" t="inlineStr">
         <is>
-          <t>Wants online menu + call button. Deposit paid 2026-07-21.</t>
+          <t>Portfolio piece / first build. Booking via fresha.com/a/dads-barbershop-martensville-402-1-avenue-south-aar4gsk8</t>
         </is>
       </c>
     </row>
@@ -7504,7 +7448,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -7543,7 +7486,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Delete the yellow-highlighted EXAMPLE row on the Pipeline tab before entering real leads.</t>
+          <t>Row 3 already has Dad's Barbershop as your first entry / portfolio piece.</t>
         </is>
       </c>
     </row>
@@ -7555,7 +7498,7 @@
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Add one row per business. Fill Business Info + Date Added + Status = New Lead as soon as you find them.</t>
+          <t>Add one new row per business. Fill Business Info + Date Added + Status = New Lead as soon as you find them.</t>
         </is>
       </c>
     </row>
@@ -7567,7 +7510,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Update Status as things move. The row's color changes automatically.</t>
+          <t>Update Status as things move. The row's Status cell color changes automatically.</t>
         </is>
       </c>
     </row>

</xml_diff>